<commit_message>
fix(pricing-calibration): calibrate synthetic prices against real-world retail benchmarks across all 16 SKUs
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -520,16 +520,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>121</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SMA-APP-IPH-121</t>
+          <t>APL-IPH16PM-256</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>8814683940853</t>
+          <t>195949038291</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Apple iPhone 5s</t>
+          <t>Apple iPhone 16 Pro Max 256GB Titanium</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -549,17 +549,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/iphone-5s/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1695048133142-1a20484d2569?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>143.99</v>
+        <v>990</v>
       </c>
       <c r="I2" t="n">
-        <v>199.99</v>
+        <v>1199</v>
       </c>
       <c r="J2" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -573,18 +573,18 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Apple iPhone 5s Smartphone (Unlocked)</t>
+          <t>Apple iPhone 16 Pro Max (256GB) - Natural Titanium</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>203.99</v>
+        <v>1189.99</v>
       </c>
       <c r="O2" t="b">
         <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>B0000121X</t>
+          <t>B0DGJQM56X</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -594,11 +594,11 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>iPhone 5s - Apple Edition</t>
+          <t>Apple - iPhone 16 Pro Max 256GB - Titanium</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>191.99</v>
+        <v>1194</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -606,16 +606,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>122</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SMA-APP-IPH-122</t>
+          <t>APL-IPH15P-128</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9922357685013</t>
+          <t>195949012384</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Apple iPhone 6</t>
+          <t>Apple iPhone 15 Pro 128GB Blue Titanium</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -635,17 +635,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/iphone-6/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1592750475338-74b7b21085ab?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>215.99</v>
+        <v>680</v>
       </c>
       <c r="I3" t="n">
-        <v>299.99</v>
+        <v>869.99</v>
       </c>
       <c r="J3" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -659,18 +659,18 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Apple iPhone 6 Smartphone (Unlocked)</t>
+          <t>Apple iPhone 15 Pro, 128GB, Blue Titanium - Unlocked</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>299.99</v>
+        <v>829.99</v>
       </c>
       <c r="O3" t="b">
         <v>1</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>B0000122X</t>
+          <t>B0CHWZ6R2X</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -680,11 +680,11 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>iPhone 6 - Apple Edition</t>
+          <t>Apple - iPhone 15 Pro 128GB - Blue Titanium (Unlocked)</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>299.99</v>
+        <v>849.99</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -692,16 +692,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>123</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SMA-APP-IPH-123</t>
+          <t>APL-MBA15-M3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4998438802308</t>
+          <t>195949112233</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -711,27 +711,27 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Apple iPhone 13 Pro</t>
+          <t>Apple MacBook Air 15" M3 512GB Midnight</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Laptops</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/iphone-13-pro/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1517336714731-489689fd1ca8?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>791.99</v>
+        <v>1080</v>
       </c>
       <c r="I4" t="n">
-        <v>1099.99</v>
+        <v>1399</v>
       </c>
       <c r="J4" t="n">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -745,18 +745,18 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Apple iPhone 13 Pro Smartphone (Unlocked)</t>
+          <t>Apple 2024 MacBook Air 15-inch Laptop with M3 chip, 512GB</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>1084.99</v>
+        <v>1299</v>
       </c>
       <c r="O4" t="b">
         <v>1</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>B0000123X</t>
+          <t>B0CX2345M3</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -766,11 +766,11 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>iPhone 13 Pro - Apple Edition</t>
+          <t>MacBook Air 15" Laptop - M3 chip - 512GB SSD - Midnight</t>
         </is>
       </c>
       <c r="S4" t="n">
-        <v>1104.99</v>
+        <v>1349</v>
       </c>
       <c r="T4" t="b">
         <v>1</v>
@@ -778,16 +778,16 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>124</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SMA-APP-IPH-124</t>
+          <t>APL-APMAX-USBC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3034949322264</t>
+          <t>195949887766</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -797,27 +797,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Apple iPhone X</t>
+          <t>Apple AirPods Max (USB-C) Space Gray</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/iphone-x/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1546435770-a3e426bf472b?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>647.99</v>
+        <v>410</v>
       </c>
       <c r="I5" t="n">
-        <v>899.99</v>
+        <v>549</v>
       </c>
       <c r="J5" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -831,18 +831,18 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Apple iPhone X Smartphone (Unlocked)</t>
+          <t>Apple AirPods Max Wireless Over-Ear Headphones, USB-C</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>884.99</v>
+        <v>499</v>
       </c>
       <c r="O5" t="b">
         <v>1</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>B0000124X</t>
+          <t>B0DGJMAX88</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -852,11 +852,11 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>iPhone X - Apple Edition</t>
+          <t>Apple - AirPods Max (USB-C) - Space Gray</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>911.99</v>
+        <v>529</v>
       </c>
       <c r="T5" t="b">
         <v>1</v>
@@ -864,46 +864,46 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>125</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SMA-OPP-OPP-125</t>
+          <t>APL-IPADP13-M4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0651223722522</t>
+          <t>195949221100</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Oppo</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Oppo Oppo A57</t>
+          <t>Apple iPad Pro 13" M4 OLED 256GB Silver</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Tablets</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/oppo-a57/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1544244015-0df4b3ffc6b0?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>179.99</v>
+        <v>990</v>
       </c>
       <c r="I6" t="n">
-        <v>249.99</v>
+        <v>1299</v>
       </c>
       <c r="J6" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -917,18 +917,18 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Oppo Oppo A57 Smartphone (Unlocked)</t>
+          <t>Apple iPad Pro 13-Inch (M4): Ultra Retina XDR Display, 256GB</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>244.99</v>
+        <v>1199</v>
       </c>
       <c r="O6" t="b">
         <v>1</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>B0000125X</t>
+          <t>B0D3J13M4P</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -938,11 +938,11 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Oppo A57 - Oppo Edition</t>
+          <t>Apple - 13-Inch iPad Pro (M4) with Wi-Fi 256GB - Silver</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>249.99</v>
+        <v>1249</v>
       </c>
       <c r="T6" t="b">
         <v>1</v>
@@ -950,26 +950,26 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>126</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SMA-OPP-OPP-126</t>
+          <t>SAM-S24U-512</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8576893968169</t>
+          <t>887276812345</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Oppo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Oppo Oppo F19 Pro Plus</t>
+          <t>Samsung Galaxy S24 Ultra 512GB Titanium Gray</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -979,17 +979,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/oppo-f19-pro-plus/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1610945265064-0e34e5519bbf?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>287.99</v>
+        <v>950</v>
       </c>
       <c r="I7" t="n">
-        <v>399.99</v>
+        <v>1219.99</v>
       </c>
       <c r="J7" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1003,18 +1003,18 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Oppo Oppo F19 Pro Plus Smartphone (Unlocked)</t>
+          <t>SAMSUNG Galaxy S24 Ultra Cell Phone 512GB AI Smartphone</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>399.99</v>
+        <v>1149.99</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>B0000126X</t>
+          <t>B0CQY8S24U</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1024,11 +1024,11 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Oppo F19 Pro Plus - Oppo Edition</t>
+          <t>Samsung - Galaxy S24 Ultra 512GB (Unlocked) - Titanium Gray</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>399.99</v>
+        <v>1179.99</v>
       </c>
       <c r="T7" t="b">
         <v>1</v>
@@ -1036,26 +1036,26 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>127</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SMA-OPP-OPP-127</t>
+          <t>SAM-ZFOLD6-256</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3106827888743</t>
+          <t>887276899887</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Oppo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Oppo Oppo K1</t>
+          <t>Samsung Galaxy Z Fold 6 256GB Silver Shadow</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1065,17 +1065,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/oppo-k1/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1580910051074-3eb694886505?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>215.99</v>
+        <v>1320</v>
       </c>
       <c r="I8" t="n">
-        <v>299.99</v>
+        <v>1699.99</v>
       </c>
       <c r="J8" t="n">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1089,18 +1089,18 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Oppo Oppo K1 Smartphone (Unlocked)</t>
+          <t>SAMSUNG Galaxy Z Fold 6 AI Cell Phone, 256GB Unlocked</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>309.99</v>
+        <v>1599.99</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>B0000127X</t>
+          <t>B0D6FZFOLD</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1110,11 +1110,11 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Oppo K1 - Oppo Edition</t>
+          <t>Samsung - Galaxy Z Fold6 256GB (Unlocked) - Silver Shadow</t>
         </is>
       </c>
       <c r="S8" t="n">
-        <v>304.99</v>
+        <v>1649.99</v>
       </c>
       <c r="T8" t="b">
         <v>1</v>
@@ -1122,46 +1122,46 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SMA-REA-REA-128</t>
+          <t>SAM-GWULTRA-47</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>7825844344364</t>
+          <t>887276844556</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Realme</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Realme Realme C35</t>
+          <t>Samsung Galaxy Watch Ultra 47mm LTE Titanium</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Wearables</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/realme-c35/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1523275335684-37898b6baf30?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>107.99</v>
+        <v>450</v>
       </c>
       <c r="I9" t="n">
-        <v>149.99</v>
+        <v>649.99</v>
       </c>
       <c r="J9" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1175,18 +1175,18 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Realme Realme C35 Smartphone (Unlocked)</t>
+          <t>SAMSUNG Galaxy Watch Ultra 47mm LTE AI Smartwatch Titanium</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>153.99</v>
+        <v>549.99</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>B0000128X</t>
+          <t>B0D7GWULTR</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1196,11 +1196,11 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Realme C35 - Realme Edition</t>
+          <t>Samsung - Galaxy Watch Ultra Titanium Smartwatch 47mm LTE</t>
         </is>
       </c>
       <c r="S9" t="n">
-        <v>149.99</v>
+        <v>599.99</v>
       </c>
       <c r="T9" t="b">
         <v>1</v>
@@ -1208,46 +1208,46 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>129</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SMA-REA-REA-129</t>
+          <t>SNY-WH1000XM5-B</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>4948452391831</t>
+          <t>027242923456</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Realme</t>
+          <t>Sony</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Realme Realme X</t>
+          <t>Sony WH-1000XM5 Wireless ANC Headphones</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/realme-x/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1505740420928-5e560c06d30e?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>215.99</v>
+        <v>265</v>
       </c>
       <c r="I10" t="n">
-        <v>299.99</v>
+        <v>379.99</v>
       </c>
       <c r="J10" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1261,18 +1261,18 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Realme Realme X Smartphone (Unlocked)</t>
+          <t>Sony WH-1000XM5 Wireless Industry Leading Noise Canceling</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>299.99</v>
+        <v>328</v>
       </c>
       <c r="O10" t="b">
         <v>1</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>B0000129X</t>
+          <t>B09XS7JWHH</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1282,58 +1282,58 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Realme X - Realme Edition</t>
+          <t>Sony - WH-1000XM5 Wireless Noise-Canceling Headphones</t>
         </is>
       </c>
       <c r="S10" t="n">
-        <v>299.99</v>
+        <v>348</v>
       </c>
       <c r="T10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SMA-REA-REA-130</t>
+          <t>SNY-PS5PRO-2TB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>6151817227632</t>
+          <t>711719582234</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Realme</t>
+          <t>Sony</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Realme Realme XT</t>
+          <t>Sony PlayStation 5 Pro Console 2TB SSD</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Gaming</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/realme-xt/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1606813907291-d86efa9b94db?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>251.99</v>
+        <v>590</v>
       </c>
       <c r="I11" t="n">
-        <v>349.99</v>
+        <v>699.99</v>
       </c>
       <c r="J11" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1347,18 +1347,18 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Realme Realme XT Smartphone (Unlocked)</t>
+          <t>PlayStation 5 Pro Console (2TB)</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>334.99</v>
+        <v>699.99</v>
       </c>
       <c r="O11" t="b">
         <v>1</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>B0000130X</t>
+          <t>B0DFPS5PRO</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1368,11 +1368,11 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Realme XT - Realme Edition</t>
+          <t>Sony - PlayStation 5 Pro Console - White</t>
         </is>
       </c>
       <c r="S11" t="n">
-        <v>349.99</v>
+        <v>699.99</v>
       </c>
       <c r="T11" t="b">
         <v>1</v>
@@ -1380,46 +1380,46 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>131</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SMA-SAM-SAM-131</t>
+          <t>DYS-AIRWRAP-CMP</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>7557912146622</t>
+          <t>885609028888</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Dyson</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S7</t>
+          <t>Dyson Airwrap Multi-Styler Complete Long</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Beauty Tech</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/samsung-galaxy-s7/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1522337360788-8b13dee7a37e?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>215.99</v>
+        <v>470</v>
       </c>
       <c r="I12" t="n">
-        <v>299.99</v>
+        <v>599.99</v>
       </c>
       <c r="J12" t="n">
-        <v>67</v>
+        <v>16</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1433,18 +1433,18 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S7 Smartphone (Unlocked)</t>
+          <t>Dyson Airwrap Multi-Styler Complete Long, Nickel/Copper</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>303.99</v>
+        <v>579.99</v>
       </c>
       <c r="O12" t="b">
         <v>1</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>B0000131X</t>
+          <t>B09YAIRWRP</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1454,11 +1454,11 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S7 - Samsung Edition</t>
+          <t>Dyson - Airwrap Multi-Styler Complete Long - Nickel/Copper</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>299.99</v>
+        <v>589.99</v>
       </c>
       <c r="T12" t="b">
         <v>1</v>
@@ -1466,50 +1466,50 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>132</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SMA-SAM-SAM-132</t>
+          <t>DYS-V15-DETECT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>5995499013336</t>
+          <t>885609017777</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Dyson</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S8</t>
+          <t>Dyson V15 Detect Cordless Vacuum Yellow/Iron</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Home Appliances</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/samsung-galaxy-s8/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1558317374-067fb5f30001?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>359.99</v>
+        <v>530</v>
       </c>
       <c r="I13" t="n">
-        <v>499.99</v>
+        <v>749.99</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Out of Stock</t>
+          <t>In Stock</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1519,18 +1519,18 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S8 Smartphone (Unlocked)</t>
+          <t>Dyson V15 Detect Cordless Vacuum Cleaner, Yellow/Iron</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>499.99</v>
+        <v>649.99</v>
       </c>
       <c r="O13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>B0000132X</t>
+          <t>B094V15DET</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1540,55 +1540,55 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S8 - Samsung Edition</t>
+          <t>Dyson - V15 Detect Cordless Vacuum - Yellow/Iron</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>511.99</v>
+        <v>699.99</v>
       </c>
       <c r="T13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>133</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SMA-SAM-SAM-133</t>
+          <t>BSE-QCU-BLK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4676898229465</t>
+          <t>017817844332</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Audio / Gadgets</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S10</t>
+          <t>Bose QuietComfort Ultra Headphones Black</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/samsung-galaxy-s10/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1546435770-a3e426bf472b?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>503.99</v>
+        <v>310</v>
       </c>
       <c r="I14" t="n">
-        <v>699.99</v>
+        <v>429</v>
       </c>
       <c r="J14" t="n">
         <v>19</v>
@@ -1605,18 +1605,18 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Samsung Samsung Galaxy S10 Smartphone (Unlocked)</t>
+          <t>Bose QuietComfort Ultra Wireless Noise Cancelling Headphones</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>684.99</v>
+        <v>379</v>
       </c>
       <c r="O14" t="b">
         <v>1</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>B0000133X</t>
+          <t>B0CCZ26BSE</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1626,11 +1626,11 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S10 - Samsung Edition</t>
+          <t>Bose - QuietComfort Ultra Wireless Headphones - Black</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>704.99</v>
+        <v>399</v>
       </c>
       <c r="T14" t="b">
         <v>1</v>
@@ -1638,26 +1638,26 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>134</v>
+        <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SMA-VIV-VIV-134</t>
+          <t>GGL-PX9PXL-256</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8575699153333</t>
+          <t>840244701234</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Vivo</t>
+          <t>Audio / Gadgets</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Vivo Vivo S1</t>
+          <t>Google Pixel 9 Pro XL 256GB Obsidian</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1667,17 +1667,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/vivo-s1/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1598327105666-5b89351aff97?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>179.99</v>
+        <v>860</v>
       </c>
       <c r="I15" t="n">
-        <v>249.99</v>
+        <v>1149</v>
       </c>
       <c r="J15" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1691,18 +1691,18 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Vivo Vivo S1 Smartphone (Unlocked)</t>
+          <t>Google Pixel 9 Pro XL - Unlocked Android Smartphone - 256 GB</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>249.99</v>
+        <v>1049</v>
       </c>
       <c r="O15" t="b">
         <v>1</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>B0000134X</t>
+          <t>B0D8PX9PXL</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Vivo S1 - Vivo Edition</t>
+          <t>Google - Pixel 9 Pro XL 256GB (Unlocked) - Obsidian</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>241.99</v>
+        <v>1069</v>
       </c>
       <c r="T15" t="b">
         <v>1</v>
@@ -1724,46 +1724,46 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>135</v>
+        <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SMA-VIV-VIV-135</t>
+          <t>DJI-MINI4P-FMC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>4295398764784</t>
+          <t>190021008765</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Vivo</t>
+          <t>Audio / Gadgets</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Vivo Vivo V9</t>
+          <t>DJI Mini 4 Pro Drone Fly More Combo RC 2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>Drones</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/vivo-v9/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1508614589041-895b88991e3e?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>215.99</v>
+        <v>860</v>
       </c>
       <c r="I16" t="n">
-        <v>299.99</v>
+        <v>1099</v>
       </c>
       <c r="J16" t="n">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1777,18 +1777,18 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Vivo Vivo V9 Smartphone (Unlocked)</t>
+          <t>DJI Mini 4 Pro Fly More Combo with RC 2 Remote Controller</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>303.99</v>
+        <v>1049</v>
       </c>
       <c r="O16" t="b">
         <v>1</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>B0000135X</t>
+          <t>B0CGLMINI4</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1798,11 +1798,11 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Vivo V9 - Vivo Edition</t>
+          <t>DJI - Mini 4 Pro Fly More Combo with RC 2 Controller</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>299.99</v>
+        <v>1079</v>
       </c>
       <c r="T16" t="b">
         <v>1</v>
@@ -1810,46 +1810,46 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>136</v>
+        <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SMA-VIV-VIV-136</t>
+          <t>MTA-QUEST3-512</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>9944308291810</t>
+          <t>815820023456</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Vivo</t>
+          <t>Audio / Gadgets</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Vivo Vivo X21</t>
+          <t>Meta Quest 3 512GB Breakthrough Mixed Reality</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Smartphones</t>
+          <t>VR / AR</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://cdn.dummyjson.com/product-images/smartphones/vivo-x21/thumbnail.webp</t>
+          <t>https://images.unsplash.com/photo-1622979135225-d2ba269bc1df?w=150&amp;auto=format&amp;fit=crop&amp;q=80</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>359.99</v>
+        <v>395</v>
       </c>
       <c r="I17" t="n">
         <v>499.99</v>
       </c>
       <c r="J17" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1863,18 +1863,18 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Vivo Vivo X21 Smartphone (Unlocked)</t>
+          <t>Meta Quest 3 512GB - Advanced All-In-One VR Headset</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>484.99</v>
+        <v>489.99</v>
       </c>
       <c r="O17" t="b">
         <v>1</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>B0000136X</t>
+          <t>B0C8VKMTA3</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1884,14 +1884,14 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Vivo X21 - Vivo Edition</t>
+          <t>Meta - Quest 3 512GB All-in-One VR Headset</t>
         </is>
       </c>
       <c r="S17" t="n">
         <v>499.99</v>
       </c>
       <c r="T17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(benchmark): align Galaxy Z Fold 6 price with live Amazon price (1749 EUR/1729 USD)
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1320</v>
+        <v>1400</v>
       </c>
       <c r="I8" t="n">
-        <v>1699.99</v>
+        <v>1799.99</v>
       </c>
       <c r="J8" t="n">
         <v>14</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>1599.99</v>
+        <v>1729</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>1649.99</v>
+        <v>1749.99</v>
       </c>
       <c r="T8" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
fix(calibration): set Fold 6 to 2026 street price ,099.99 matching live Amazon new sale benchmarks
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1400</v>
+        <v>890</v>
       </c>
       <c r="I8" t="n">
-        <v>1799.99</v>
+        <v>1199.99</v>
       </c>
       <c r="J8" t="n">
         <v>14</v>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>1729</v>
+        <v>1099.99</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>1749.99</v>
+        <v>1149.99</v>
       </c>
       <c r="T8" t="b">
         <v>1</v>

</xml_diff>